<commit_message>
Static variable renaming in Node/Node.cpp + Autogen DataBlock NUMBER_OF_VARS change
</commit_message>
<xml_diff>
--- a/Documentation/Universal Data Block Definitions.xlsx
+++ b/Documentation/Universal Data Block Definitions.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
   <si>
     <t xml:space="preserve">Var ID</t>
   </si>
@@ -47,13 +47,17 @@
 Reset Node</t>
   </si>
   <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
     <t xml:space="preserve">Configuration Status</t>
   </si>
   <si>
     <t xml:space="preserve">See ConfigurationStates_t in AtamsTypedef.hpp for possible values.
 A value of 0 indicates that the configuration state is inactive. Write access to the Universal Data Block registers is blocked.
 A value of 1 indicates that the configuration state is active. Write access to the Universal Data Block registers is allowed.
-A value of 3 indicates that the configuration state is denied. The request to enter the configuration state was denied by the Node (see Configuration Passkey). Write access to the Universal Data Block registers is blocked. </t>
+A value of 3 indicates that the configuration state is denied. The request to enter the configuration state was denied by the Node (see Configuration Passkey). Write access to the Universal Data Block registers is blocked. 
+If the Configuration Status is read in the same Atams Request Packet as a Configuration Passkey write, the Configuration Status will not reflect any actions taken due to the Configuration Passkey change.</t>
   </si>
   <si>
     <t xml:space="preserve">Store All</t>
@@ -83,25 +87,87 @@
     <t xml:space="preserve">Storage Error</t>
   </si>
   <si>
-    <t xml:space="preserve">Holds the Atams::Error_t status of the last called storage process, including Store All, Restore User Blocks, and Restore All. If the last storage process has finished (see Storage Process Complete) and the value of Storage Status is equal to Atams::ERROR_NONE, the storage process was successful. Storage Status will show as pending whilst a storage process is in progress.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Storage State</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holds a value of 1 if the last requested storage process has finished, otherwise holds a value of 0. Storage Process Complete will hold a value of 1 after a node reset, as a load process is called during initialisation.</t>
+    <t xml:space="preserve">Holds the Atams::Error_t status of the last called storage process, including Store All, Restore User Blocks, and Restore All.
+If the last storage process has finished (see Storage Process Complete) and the value of Storage Status is equal to Atams::ERROR_NONE, the storage process was successful.
+The Storage Error register can be read after Node initialisation to check the validity of the NVM storage - a load process is called during initialisation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storage Process Complete</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Holds a value of 1 if the last requested storage process has finished, otherwise holds a value of 0. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Reading the Storage Process Complete register will clear it’s value to 0. It is recommended to read the Storage State to clear the value before starting a storage process. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFC9211E"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Once a storage process has been triggered, the Node will not respond to subsequent request messages until the storage process is complete. If the storage process is successfully triggered, the Storage Process Complete register will hold a value of 1 on the first read once the Node responses return. The register will hold a value of 0 if the storage process was not triggered correctly.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">If the Storage Status is read in the same Atams Request Packet as a store/restore passcode write, the Storage Status will not reflect any actions taken from the the store/restore passcode change.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Storage Process Complete will hold a value of 1 after a node reset – a load process is called during initialisation.</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Watchdog Fault Active</t>
   </si>
   <si>
-    <t xml:space="preserve">The communications watchdog will trigger a fault if the time between request messages received from the Atams Hub has exceeded the watchdog period. Watchdog Fault Active will hold a value of 1 if the watchdog the period has been exceeded and the watchdog fault is active. A value of 0 indicates the watchdog fault is inactive.</t>
+    <t xml:space="preserve">The communications watchdog will trigger a fault if the time between request messages received from the Atams Hub exceeds the watchdog period. Watchdog Fault Active will hold a value of 1 if the watchdog period has been exceeded and the watchdog fault is active. A value of 0 indicates the watchdog fault is inactive.</t>
   </si>
   <si>
     <t xml:space="preserve">Watchdog Reset</t>
   </si>
   <si>
-    <t xml:space="preserve">The watchdog fault will be cleared when a value of FILLMEIN is written to the Watchdog Reset register and the previous value held in the Watchdog Reset register is 0.</t>
+    <t xml:space="preserve">The watchdog fault will be cleared when a value of FILLMEIN is written to the Watchdog Reset register and the previous value held in the Watchdog Reset register is not equal to FILLMEIN.</t>
   </si>
 </sst>
 </file>
@@ -112,11 +178,12 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -135,6 +202,26 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC9211E"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -182,28 +269,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -211,7 +302,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -224,6 +315,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FFC9211E"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -338,220 +489,250 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="73.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="73.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="304.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="126.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="171.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
+      <c r="B3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="35.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="B4" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="46.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
+      <c r="B5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="46.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
+      <c r="B6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="57.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="B7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C7" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="92.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="35.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="B8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C8" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="206.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
         <v>17</v>
       </c>
+      <c r="B9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="46.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="B10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C10" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="35.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
         <v>21</v>
       </c>
+      <c r="B11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
+      <c r="A27" s="8"/>
+      <c r="B27" s="8"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
+      <c r="A35" s="8"/>
+      <c r="B35" s="8"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
+      <c r="A38" s="8"/>
+      <c r="B38" s="8"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
+      <c r="A39" s="8"/>
+      <c r="B39" s="8"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
+      <c r="A40" s="8"/>
+      <c r="B40" s="8"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
+      <c r="A41" s="8"/>
+      <c r="B41" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Part way through bus updates Hub. Pre DataBlock removal.
</commit_message>
<xml_diff>
--- a/Documentation/Universal Data Block Definitions.xlsx
+++ b/Documentation/Universal Data Block Definitions.xlsx
@@ -135,26 +135,9 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Once a storage process has been triggered, the Node will not respond to subsequent request messages until the storage process is complete. If the storage process is successfully triggered, the Storage Process Complete register will hold a value of 1 on the first read once the Node responses return. The register will hold a value of 0 if the storage process was not triggered correctly.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">If the Storage Status is read in the same Atams Request Packet as a store/restore passcode write, the Storage Status will not reflect any actions taken from the the store/restore passcode change.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Storage Process Complete will hold a value of 1 after a node reset – a load process is called during initialisation.</t>
+      <t xml:space="preserve">Once a storage process has been triggered and the passcode assess has been acknowledged, the Node will not respond to subsequent request messages until the storage process is complete. If the storage process is successfully triggered, the Storage Process Complete register will hold a value of 1 on the first successful read once the Node responses return. The register will hold a value of 0 if the storage process was not triggered correctly.
+If the Storage Status is read in the same Atams Request Packet as a store/restore passcode write, the Storage Status will not reflect any actions taken from the the store/restore passcode change.
+Storage Process Complete will hold a value of 1 after a node reset – a load process is called during initialisation.</t>
     </r>
   </si>
   <si>
@@ -178,7 +161,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -220,11 +203,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -581,7 +559,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="206.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="217.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Bug fix - following nodes ignored if response of previous node timed out
</commit_message>
<xml_diff>
--- a/Documentation/Universal Data Block Definitions.xlsx
+++ b/Documentation/Universal Data Block Definitions.xlsx
@@ -56,7 +56,8 @@
     <t xml:space="preserve">See ConfigurationStates_t in AtamsTypedef.hpp for possible values.
 A value of 0 indicates that the configuration state is inactive. Write access to the Universal Data Block registers is blocked.
 A value of 1 indicates that the configuration state is active. Write access to the Universal Data Block registers is allowed.
-A value of 3 indicates that the configuration state is denied. The request to enter the configuration state was denied by the Node (see Configuration Passkey). Write access to the Universal Data Block registers is blocked. 
+A value of 2 indicates that the configuration state is denied. The request to enter the configuration state was denied by the Node (see Configuration Passkey). Write access to the Universal Data Block registers is blocked. 
+A value of 3 indicates the configuration has been successfully applied.
 If the Configuration Status is read in the same Atams Request Packet as a Configuration Passkey write, the Configuration Status will not reflect any actions taken due to the Configuration Passkey change.</t>
   </si>
   <si>
@@ -493,7 +494,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="171.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="194.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
         <v>5</v>
       </c>

</xml_diff>